<commit_message>
Tagueamento: canais reais com plataforma (APP/WEB)
App Sicredi e Sicredi X = APP; Internet Banking, Internet Banking PJ e
Internet Banking - Plataforma = WEB (confirmado pelo Mau). O template de
exemplo passa a usar o canal real "Internet Banking - Plataforma".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVbhaTtaKirJEjgzhEqDq7
</commit_message>
<xml_diff>
--- a/src/tagueamento/data/regions.template.xlsx
+++ b/src/tagueamento/data/regions.template.xlsx
@@ -606,7 +606,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>[EXEMPLO] Internet Banking</t>
+          <t>Internet Banking - Plataforma</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -633,7 +633,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>[EXEMPLO] Internet Banking</t>
+          <t>Internet Banking - Plataforma</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -660,7 +660,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>[EXEMPLO] Internet Banking</t>
+          <t>Internet Banking - Plataforma</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">

</xml_diff>